<commit_message>
Updated BIFUbC, removed extraneous files, ran CSV exporter
</commit_message>
<xml_diff>
--- a/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
+++ b/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ccs\NBICP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\ccs\NBICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4527F4-06B7-435E-8932-6A478272C4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E243723-5BA1-4981-9C22-BBBBBAB92F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-4770" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Capacity Factor Data" sheetId="20" r:id="rId3"/>
     <sheet name="Current and Planned Capacity" sheetId="17" r:id="rId4"/>
     <sheet name="BAU Emissions" sheetId="21" r:id="rId5"/>
-    <sheet name="BBICP-CS" sheetId="22" r:id="rId6"/>
+    <sheet name="NBICP-CS" sheetId="22" r:id="rId6"/>
     <sheet name="NBICP-FoCPAbI-energyEmis" sheetId="18" r:id="rId7"/>
     <sheet name="NBICP-FoCPAbI-processEmis" sheetId="16" r:id="rId8"/>
   </sheets>
@@ -2058,30 +2058,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="103.42578125" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="103.453125" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="22.1796875" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -2089,75 +2089,75 @@
         <v>162</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="8">
         <v>2023</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" s="9" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" s="9"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" s="10" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" s="8">
         <v>2022</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B16" s="37" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B19" s="10" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B20" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B21" s="8">
         <v>2019</v>
       </c>
@@ -2165,66 +2165,66 @@
       <c r="D21" s="3"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B22" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B23" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="2"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B24" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B25" s="8"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>34</v>
       </c>
       <c r="B32" s="1"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>173</v>
       </c>
@@ -2242,20 +2242,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9816DDC5-B47D-412D-83A1-985DCFECCE82}">
   <dimension ref="A1:I48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="47.7109375" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
-    <col min="4" max="4" width="27.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="8" customWidth="1"/>
-    <col min="6" max="6" width="30.140625" customWidth="1"/>
-    <col min="7" max="7" width="26.28515625" customWidth="1"/>
-    <col min="8" max="8" width="37.28515625" customWidth="1"/>
-    <col min="9" max="9" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="47.7265625" customWidth="1"/>
+    <col min="2" max="2" width="25.7265625" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" customWidth="1"/>
+    <col min="4" max="4" width="27.81640625" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="30.1796875" customWidth="1"/>
+    <col min="7" max="7" width="26.26953125" customWidth="1"/>
+    <col min="8" max="8" width="37.26953125" customWidth="1"/>
+    <col min="9" max="9" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
         <v>115</v>
       </c>
@@ -2268,7 +2268,7 @@
       <c r="H1" s="20"/>
       <c r="I1" s="20"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>114</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>106</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>105</v>
       </c>
@@ -2340,7 +2340,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>104</v>
       </c>
@@ -2363,7 +2363,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>103</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>102</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>98</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>97</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>95</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="87" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>94</v>
       </c>
@@ -2524,7 +2524,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>91</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>90</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>85</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>84</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>81</v>
       </c>
@@ -2665,7 +2665,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>78</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>77</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>75</v>
       </c>
@@ -2737,7 +2737,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>72</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>70</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>63</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>59</v>
       </c>
@@ -2872,7 +2872,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>57</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>54</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>53</v>
       </c>
@@ -2941,13 +2941,13 @@
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="16" t="s">
         <v>47</v>
       </c>
       <c r="B34" s="15"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>46</v>
       </c>
@@ -2956,7 +2956,7 @@
         <v>28.360000000000003</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -2965,13 +2965,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="14" t="s">
         <v>44</v>
       </c>
       <c r="B39" s="13"/>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>0.6921272158498436</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>4.6923879040667367E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -3010,7 +3010,7 @@
         <v>7.8206465067778938E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>40</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>5.7351407716371226E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>39</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>3.6496350364963501E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>38</v>
       </c>
@@ -3049,7 +3049,7 @@
         <v>2.0855057351407719E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>37</v>
       </c>
@@ -3062,7 +3062,7 @@
         <v>3.6235662148070912E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>36</v>
       </c>
@@ -3075,7 +3075,7 @@
         <v>5.7351407716371219E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>35</v>
       </c>
@@ -3105,30 +3105,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED05A5AB-C865-4DF5-BD35-041C1CC241DD}">
   <dimension ref="A1:H48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="24.1796875" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="10.453125" customWidth="1"/>
+    <col min="4" max="4" width="20.26953125" customWidth="1"/>
+    <col min="5" max="5" width="19.54296875" customWidth="1"/>
+    <col min="6" max="6" width="14.54296875" customWidth="1"/>
+    <col min="7" max="7" width="17.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>151</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2000</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -3166,19 +3166,19 @@
         <v>150</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>149</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="36" t="s">
         <v>147</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="34">
         <v>0.56999999999999995</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="34">
         <v>0.34</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="34">
         <v>0.03</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="34">
         <v>0.03</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="34">
         <v>0.02</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="34">
         <v>0.04</v>
       </c>
@@ -3261,49 +3261,49 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B18" s="5"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="34">
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="34" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>136</v>
       </c>
       <c r="B24" s="5"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>70</v>
       </c>
@@ -3311,12 +3311,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>80</v>
       </c>
@@ -3324,12 +3324,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <f>B5*B12</f>
         <v>82.524271844660205</v>
@@ -3338,8 +3338,8 @@
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="33" t="s">
         <v>128</v>
       </c>
@@ -3350,7 +3350,7 @@
       <c r="F33" s="32"/>
       <c r="G33" s="31"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="28"/>
       <c r="B34" s="29" t="s">
         <v>127</v>
@@ -3374,7 +3374,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="28" t="s">
         <v>121</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>167.47572815533979</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="28" t="s">
         <v>120</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>33.486929491831802</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="26" t="s">
         <v>119</v>
       </c>
@@ -3462,37 +3462,37 @@
         <v>57.76699029126214</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C38" s="2"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42">
         <f>'Operational Capacity'!B35</f>
         <v>28.360000000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="12">
         <f>C36/A42</f>
         <v>0.87296479384337322</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="3">
         <f>A45*'Operational Capacity'!B36</f>
         <v>8.7296479384337324</v>
@@ -3506,12 +3506,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{000817FC-5CAD-42B5-92F8-1A675198574D}">
   <dimension ref="A25:H54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="48.28515625" customWidth="1"/>
+    <col min="1" max="1" width="48.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>170</v>
       </c>
@@ -3523,7 +3523,7 @@
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B26">
         <v>2022</v>
       </c>
@@ -3534,17 +3534,17 @@
         <v>2035</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>3</v>
       </c>
@@ -3558,32 +3558,32 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>174</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>175</v>
       </c>
@@ -3617,7 +3617,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>10</v>
       </c>
@@ -3625,17 +3625,17 @@
         <v>176</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>14</v>
       </c>
@@ -3663,62 +3663,62 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>122</v>
       </c>
@@ -3744,17 +3744,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D869D793-4D45-441A-BEF3-5973BA28AC13}">
   <dimension ref="A1:AE300"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="80.140625" customWidth="1"/>
+    <col min="1" max="1" width="80.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>171</v>
       </c>
@@ -3849,7 +3849,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>178</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>9716000000000</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>179</v>
       </c>
@@ -4039,7 +4039,7 @@
         <v>665338000000</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>180</v>
       </c>
@@ -4134,7 +4134,7 @@
         <v>69366600000000</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>181</v>
       </c>
@@ -4229,7 +4229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>182</v>
       </c>
@@ -4324,7 +4324,7 @@
         <v>6699000000000</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>183</v>
       </c>
@@ -4419,7 +4419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>184</v>
       </c>
@@ -4514,7 +4514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>185</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>75479100000000</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>187</v>
       </c>
@@ -4799,7 +4799,7 @@
         <v>160400000000000</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>188</v>
       </c>
@@ -4894,7 +4894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>189</v>
       </c>
@@ -4989,7 +4989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>190</v>
       </c>
@@ -5084,7 +5084,7 @@
         <v>83100000000000</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>191</v>
       </c>
@@ -5179,7 +5179,7 @@
         <v>44070000000000</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>192</v>
       </c>
@@ -5274,7 +5274,7 @@
         <v>5642000000000</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>193</v>
       </c>
@@ -5369,7 +5369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>194</v>
       </c>
@@ -5464,7 +5464,7 @@
         <v>546600000000</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>195</v>
       </c>
@@ -5559,7 +5559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>196</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>197</v>
       </c>
@@ -5749,7 +5749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>198</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>199</v>
       </c>
@@ -5939,7 +5939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>200</v>
       </c>
@@ -6034,7 +6034,7 @@
         <v>1400230000000</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>201</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>202</v>
       </c>
@@ -6224,7 +6224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B29" s="38"/>
       <c r="C29" s="38"/>
       <c r="D29" s="38"/>
@@ -6256,7 +6256,7 @@
       <c r="AD29" s="38"/>
       <c r="AE29" s="38"/>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>171</v>
       </c>
@@ -6351,7 +6351,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>203</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>204</v>
       </c>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>205</v>
       </c>
@@ -6636,7 +6636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>206</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>207</v>
       </c>
@@ -6826,7 +6826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>208</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>209</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>210</v>
       </c>
@@ -7111,7 +7111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>211</v>
       </c>
@@ -7206,7 +7206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>212</v>
       </c>
@@ -7301,7 +7301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>213</v>
       </c>
@@ -7396,7 +7396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>214</v>
       </c>
@@ -7491,7 +7491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>215</v>
       </c>
@@ -7586,7 +7586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>216</v>
       </c>
@@ -7681,7 +7681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>217</v>
       </c>
@@ -7776,7 +7776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>218</v>
       </c>
@@ -7871,7 +7871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>219</v>
       </c>
@@ -7966,7 +7966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>220</v>
       </c>
@@ -8061,7 +8061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>221</v>
       </c>
@@ -8156,7 +8156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>222</v>
       </c>
@@ -8251,7 +8251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>223</v>
       </c>
@@ -8346,7 +8346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>224</v>
       </c>
@@ -8441,7 +8441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>225</v>
       </c>
@@ -8536,7 +8536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>226</v>
       </c>
@@ -8631,7 +8631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>227</v>
       </c>
@@ -8726,7 +8726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>228</v>
       </c>
@@ -8821,7 +8821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>229</v>
       </c>
@@ -8916,7 +8916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>230</v>
       </c>
@@ -9011,7 +9011,7 @@
         <v>11727400000</v>
       </c>
     </row>
-    <row r="59" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>231</v>
       </c>
@@ -9106,7 +9106,7 @@
         <v>867461000000</v>
       </c>
     </row>
-    <row r="60" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>232</v>
       </c>
@@ -9201,7 +9201,7 @@
         <v>13310600000000</v>
       </c>
     </row>
-    <row r="61" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>233</v>
       </c>
@@ -9296,7 +9296,7 @@
         <v>479409000000</v>
       </c>
     </row>
-    <row r="62" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>234</v>
       </c>
@@ -9391,7 +9391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>235</v>
       </c>
@@ -9486,7 +9486,7 @@
         <v>1238280000000</v>
       </c>
     </row>
-    <row r="64" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>236</v>
       </c>
@@ -9581,7 +9581,7 @@
         <v>1923620000000</v>
       </c>
     </row>
-    <row r="65" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>237</v>
       </c>
@@ -9676,7 +9676,7 @@
         <v>5779600000000</v>
       </c>
     </row>
-    <row r="66" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>238</v>
       </c>
@@ -9771,7 +9771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>239</v>
       </c>
@@ -9866,7 +9866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>240</v>
       </c>
@@ -9961,7 +9961,7 @@
         <v>4095420000000</v>
       </c>
     </row>
-    <row r="69" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>241</v>
       </c>
@@ -10056,7 +10056,7 @@
         <v>5339520000000</v>
       </c>
     </row>
-    <row r="70" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>242</v>
       </c>
@@ -10151,7 +10151,7 @@
         <v>410773000000</v>
       </c>
     </row>
-    <row r="71" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>243</v>
       </c>
@@ -10246,7 +10246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>244</v>
       </c>
@@ -10341,7 +10341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>245</v>
       </c>
@@ -10436,7 +10436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>246</v>
       </c>
@@ -10531,7 +10531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>247</v>
       </c>
@@ -10626,7 +10626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>248</v>
       </c>
@@ -10721,7 +10721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>249</v>
       </c>
@@ -10816,7 +10816,7 @@
         <v>1496730000000</v>
       </c>
     </row>
-    <row r="78" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>250</v>
       </c>
@@ -10911,7 +10911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>251</v>
       </c>
@@ -11006,7 +11006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>252</v>
       </c>
@@ -11101,7 +11101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>253</v>
       </c>
@@ -11196,7 +11196,7 @@
         <v>6462710000000</v>
       </c>
     </row>
-    <row r="82" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>254</v>
       </c>
@@ -11291,7 +11291,7 @@
         <v>109816000000</v>
       </c>
     </row>
-    <row r="83" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>255</v>
       </c>
@@ -11386,7 +11386,7 @@
         <v>155700000000000</v>
       </c>
     </row>
-    <row r="84" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>256</v>
       </c>
@@ -11481,7 +11481,7 @@
         <v>9168770000000</v>
       </c>
     </row>
-    <row r="85" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>257</v>
       </c>
@@ -11576,7 +11576,7 @@
         <v>46034900000000</v>
       </c>
     </row>
-    <row r="86" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>258</v>
       </c>
@@ -11671,7 +11671,7 @@
         <v>6696170000000</v>
       </c>
     </row>
-    <row r="87" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>259</v>
       </c>
@@ -11766,7 +11766,7 @@
         <v>2512390000000</v>
       </c>
     </row>
-    <row r="88" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>260</v>
       </c>
@@ -11861,7 +11861,7 @@
         <v>22099500000000</v>
       </c>
     </row>
-    <row r="89" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>261</v>
       </c>
@@ -11956,7 +11956,7 @@
         <v>21011700000000</v>
       </c>
     </row>
-    <row r="90" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>262</v>
       </c>
@@ -12051,7 +12051,7 @@
         <v>146795000000000</v>
       </c>
     </row>
-    <row r="91" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>263</v>
       </c>
@@ -12146,7 +12146,7 @@
         <v>5682730000000</v>
       </c>
     </row>
-    <row r="92" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>264</v>
       </c>
@@ -12241,7 +12241,7 @@
         <v>4059090000000</v>
       </c>
     </row>
-    <row r="93" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>265</v>
       </c>
@@ -12336,7 +12336,7 @@
         <v>10214100000000</v>
       </c>
     </row>
-    <row r="94" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>266</v>
       </c>
@@ -12431,7 +12431,7 @@
         <v>18213300000000</v>
       </c>
     </row>
-    <row r="95" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>267</v>
       </c>
@@ -12526,7 +12526,7 @@
         <v>11625400000000</v>
       </c>
     </row>
-    <row r="96" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>268</v>
       </c>
@@ -12621,7 +12621,7 @@
         <v>7104730000000</v>
       </c>
     </row>
-    <row r="97" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>269</v>
       </c>
@@ -12716,7 +12716,7 @@
         <v>1530250000000</v>
       </c>
     </row>
-    <row r="98" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>270</v>
       </c>
@@ -12811,7 +12811,7 @@
         <v>2385050000000</v>
       </c>
     </row>
-    <row r="99" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>271</v>
       </c>
@@ -12906,7 +12906,7 @@
         <v>3633550000000</v>
       </c>
     </row>
-    <row r="100" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>272</v>
       </c>
@@ -13001,7 +13001,7 @@
         <v>6717400000000</v>
       </c>
     </row>
-    <row r="101" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>273</v>
       </c>
@@ -13096,7 +13096,7 @@
         <v>3802810000000</v>
       </c>
     </row>
-    <row r="102" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>274</v>
       </c>
@@ -13191,7 +13191,7 @@
         <v>20910900000000</v>
       </c>
     </row>
-    <row r="103" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>275</v>
       </c>
@@ -13286,7 +13286,7 @@
         <v>41048000000000</v>
       </c>
     </row>
-    <row r="104" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>276</v>
       </c>
@@ -13381,7 +13381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>277</v>
       </c>
@@ -13476,7 +13476,7 @@
         <v>10394500000000</v>
       </c>
     </row>
-    <row r="106" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>278</v>
       </c>
@@ -13571,7 +13571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>279</v>
       </c>
@@ -13666,7 +13666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>280</v>
       </c>
@@ -13761,7 +13761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>281</v>
       </c>
@@ -13856,7 +13856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>282</v>
       </c>
@@ -13951,7 +13951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>283</v>
       </c>
@@ -14046,7 +14046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>284</v>
       </c>
@@ -14141,7 +14141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>285</v>
       </c>
@@ -14236,7 +14236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>286</v>
       </c>
@@ -14331,7 +14331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>287</v>
       </c>
@@ -14426,7 +14426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>288</v>
       </c>
@@ -14521,7 +14521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>289</v>
       </c>
@@ -14616,7 +14616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>290</v>
       </c>
@@ -14711,7 +14711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>291</v>
       </c>
@@ -14806,7 +14806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>292</v>
       </c>
@@ -14901,7 +14901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>293</v>
       </c>
@@ -14996,7 +14996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>294</v>
       </c>
@@ -15091,7 +15091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>295</v>
       </c>
@@ -15186,7 +15186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>296</v>
       </c>
@@ -15281,7 +15281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>297</v>
       </c>
@@ -15376,7 +15376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>298</v>
       </c>
@@ -15471,7 +15471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>299</v>
       </c>
@@ -15566,7 +15566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>300</v>
       </c>
@@ -15661,7 +15661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>301</v>
       </c>
@@ -15756,7 +15756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>302</v>
       </c>
@@ -15851,7 +15851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>303</v>
       </c>
@@ -15946,7 +15946,7 @@
         <v>47012600000000</v>
       </c>
     </row>
-    <row r="132" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>304</v>
       </c>
@@ -16041,7 +16041,7 @@
         <v>560345000000</v>
       </c>
     </row>
-    <row r="133" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>305</v>
       </c>
@@ -16136,7 +16136,7 @@
         <v>9549060000000</v>
       </c>
     </row>
-    <row r="134" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>306</v>
       </c>
@@ -16231,7 +16231,7 @@
         <v>6406920000000</v>
       </c>
     </row>
-    <row r="135" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>307</v>
       </c>
@@ -16326,7 +16326,7 @@
         <v>967266000000</v>
       </c>
     </row>
-    <row r="136" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>308</v>
       </c>
@@ -16421,7 +16421,7 @@
         <v>358391000000</v>
       </c>
     </row>
-    <row r="137" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>309</v>
       </c>
@@ -16516,7 +16516,7 @@
         <v>548392000000</v>
       </c>
     </row>
-    <row r="138" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>310</v>
       </c>
@@ -16611,7 +16611,7 @@
         <v>739519000000</v>
       </c>
     </row>
-    <row r="139" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>311</v>
       </c>
@@ -16706,7 +16706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>312</v>
       </c>
@@ -16801,7 +16801,7 @@
         <v>71258000000</v>
       </c>
     </row>
-    <row r="141" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>313</v>
       </c>
@@ -16896,7 +16896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>314</v>
       </c>
@@ -16991,7 +16991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>315</v>
       </c>
@@ -17086,7 +17086,7 @@
         <v>4134700000000</v>
       </c>
     </row>
-    <row r="144" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>316</v>
       </c>
@@ -17181,7 +17181,7 @@
         <v>202683000000</v>
       </c>
     </row>
-    <row r="145" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>317</v>
       </c>
@@ -17276,7 +17276,7 @@
         <v>362743000000</v>
       </c>
     </row>
-    <row r="146" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>318</v>
       </c>
@@ -17371,7 +17371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>319</v>
       </c>
@@ -17466,7 +17466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>320</v>
       </c>
@@ -17561,7 +17561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>321</v>
       </c>
@@ -17656,7 +17656,7 @@
         <v>105131000000</v>
       </c>
     </row>
-    <row r="150" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>322</v>
       </c>
@@ -17751,7 +17751,7 @@
         <v>174318000000</v>
       </c>
     </row>
-    <row r="151" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>323</v>
       </c>
@@ -17846,7 +17846,7 @@
         <v>98602600000</v>
       </c>
     </row>
-    <row r="152" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>324</v>
       </c>
@@ -17941,7 +17941,7 @@
         <v>1119600000000</v>
       </c>
     </row>
-    <row r="153" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>325</v>
       </c>
@@ -18036,7 +18036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>326</v>
       </c>
@@ -18131,7 +18131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>327</v>
       </c>
@@ -18226,7 +18226,7 @@
         <v>42095300000000</v>
       </c>
     </row>
-    <row r="156" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>328</v>
       </c>
@@ -18321,7 +18321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>329</v>
       </c>
@@ -18416,7 +18416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>330</v>
       </c>
@@ -18511,7 +18511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>331</v>
       </c>
@@ -18606,7 +18606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>332</v>
       </c>
@@ -18701,7 +18701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>333</v>
       </c>
@@ -18796,7 +18796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>334</v>
       </c>
@@ -18891,7 +18891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>335</v>
       </c>
@@ -18986,7 +18986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>336</v>
       </c>
@@ -19081,7 +19081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>337</v>
       </c>
@@ -19176,7 +19176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>338</v>
       </c>
@@ -19271,7 +19271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>339</v>
       </c>
@@ -19366,7 +19366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>340</v>
       </c>
@@ -19461,7 +19461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>341</v>
       </c>
@@ -19556,7 +19556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>342</v>
       </c>
@@ -19651,7 +19651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>343</v>
       </c>
@@ -19746,7 +19746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>344</v>
       </c>
@@ -19841,7 +19841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>345</v>
       </c>
@@ -19936,7 +19936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>346</v>
       </c>
@@ -20031,7 +20031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>347</v>
       </c>
@@ -20126,7 +20126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>348</v>
       </c>
@@ -20221,7 +20221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>349</v>
       </c>
@@ -20316,7 +20316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>350</v>
       </c>
@@ -20411,7 +20411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>351</v>
       </c>
@@ -20506,7 +20506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>352</v>
       </c>
@@ -20601,7 +20601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>353</v>
       </c>
@@ -20696,7 +20696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>354</v>
       </c>
@@ -20791,7 +20791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>355</v>
       </c>
@@ -20886,7 +20886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>356</v>
       </c>
@@ -20981,7 +20981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>357</v>
       </c>
@@ -21076,7 +21076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>358</v>
       </c>
@@ -21171,7 +21171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>359</v>
       </c>
@@ -21266,7 +21266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>360</v>
       </c>
@@ -21361,7 +21361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>361</v>
       </c>
@@ -21456,7 +21456,7 @@
         <v>95518500000000</v>
       </c>
     </row>
-    <row r="190" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>362</v>
       </c>
@@ -21551,7 +21551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>363</v>
       </c>
@@ -21646,7 +21646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>364</v>
       </c>
@@ -21741,7 +21741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>365</v>
       </c>
@@ -21836,7 +21836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>366</v>
       </c>
@@ -21931,7 +21931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>367</v>
       </c>
@@ -22026,7 +22026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>368</v>
       </c>
@@ -22121,7 +22121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>369</v>
       </c>
@@ -22216,7 +22216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>370</v>
       </c>
@@ -22311,7 +22311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>371</v>
       </c>
@@ -22406,7 +22406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>372</v>
       </c>
@@ -22501,7 +22501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>373</v>
       </c>
@@ -22596,7 +22596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>374</v>
       </c>
@@ -22691,7 +22691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>375</v>
       </c>
@@ -22786,7 +22786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>376</v>
       </c>
@@ -22881,7 +22881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>377</v>
       </c>
@@ -22976,7 +22976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>378</v>
       </c>
@@ -23071,7 +23071,7 @@
         <v>2398450000</v>
       </c>
     </row>
-    <row r="207" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>379</v>
       </c>
@@ -23166,7 +23166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>380</v>
       </c>
@@ -23261,7 +23261,7 @@
         <v>338570000000</v>
       </c>
     </row>
-    <row r="209" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>381</v>
       </c>
@@ -23356,7 +23356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>382</v>
       </c>
@@ -23451,7 +23451,7 @@
         <v>21469000000</v>
       </c>
     </row>
-    <row r="211" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>383</v>
       </c>
@@ -23546,7 +23546,7 @@
         <v>10838400000</v>
       </c>
     </row>
-    <row r="212" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>384</v>
       </c>
@@ -23641,7 +23641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>385</v>
       </c>
@@ -23736,7 +23736,7 @@
         <v>1880500000000</v>
       </c>
     </row>
-    <row r="214" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>386</v>
       </c>
@@ -23831,7 +23831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>387</v>
       </c>
@@ -23926,7 +23926,7 @@
         <v>153739000000</v>
       </c>
     </row>
-    <row r="216" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>388</v>
       </c>
@@ -24021,7 +24021,7 @@
         <v>161615000</v>
       </c>
     </row>
-    <row r="217" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>389</v>
       </c>
@@ -24116,7 +24116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>390</v>
       </c>
@@ -24211,7 +24211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>391</v>
       </c>
@@ -24306,7 +24306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>392</v>
       </c>
@@ -24401,7 +24401,7 @@
         <v>9287170000</v>
       </c>
     </row>
-    <row r="221" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>393</v>
       </c>
@@ -24496,7 +24496,7 @@
         <v>517514</v>
       </c>
     </row>
-    <row r="222" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>394</v>
       </c>
@@ -24591,7 +24591,7 @@
         <v>2222210</v>
       </c>
     </row>
-    <row r="223" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>395</v>
       </c>
@@ -24686,7 +24686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>396</v>
       </c>
@@ -24781,7 +24781,7 @@
         <v>83436100</v>
       </c>
     </row>
-    <row r="225" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>397</v>
       </c>
@@ -24876,7 +24876,7 @@
         <v>46787300000</v>
       </c>
     </row>
-    <row r="226" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>398</v>
       </c>
@@ -24971,7 +24971,7 @@
         <v>26480300000</v>
       </c>
     </row>
-    <row r="227" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>399</v>
       </c>
@@ -25066,7 +25066,7 @@
         <v>33843400000</v>
       </c>
     </row>
-    <row r="228" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>400</v>
       </c>
@@ -25161,7 +25161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>401</v>
       </c>
@@ -25256,7 +25256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>402</v>
       </c>
@@ -25351,7 +25351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>403</v>
       </c>
@@ -25446,7 +25446,7 @@
         <v>6034760000000</v>
       </c>
     </row>
-    <row r="232" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>404</v>
       </c>
@@ -25541,7 +25541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>405</v>
       </c>
@@ -25636,7 +25636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>406</v>
       </c>
@@ -25731,7 +25731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>407</v>
       </c>
@@ -25826,7 +25826,7 @@
         <v>242521000000</v>
       </c>
     </row>
-    <row r="236" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>408</v>
       </c>
@@ -25921,7 +25921,7 @@
         <v>107125000000</v>
       </c>
     </row>
-    <row r="237" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>409</v>
       </c>
@@ -26016,7 +26016,7 @@
         <v>184319000000</v>
       </c>
     </row>
-    <row r="238" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>410</v>
       </c>
@@ -26111,7 +26111,7 @@
         <v>136687000000</v>
       </c>
     </row>
-    <row r="239" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>411</v>
       </c>
@@ -26206,7 +26206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>412</v>
       </c>
@@ -26301,7 +26301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>413</v>
       </c>
@@ -26396,7 +26396,7 @@
         <v>98336000000</v>
       </c>
     </row>
-    <row r="242" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>414</v>
       </c>
@@ -26491,7 +26491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>415</v>
       </c>
@@ -26586,7 +26586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>416</v>
       </c>
@@ -26681,7 +26681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>417</v>
       </c>
@@ -26776,7 +26776,7 @@
         <v>91821200000</v>
       </c>
     </row>
-    <row r="246" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>418</v>
       </c>
@@ -26871,7 +26871,7 @@
         <v>137978000000</v>
       </c>
     </row>
-    <row r="247" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>419</v>
       </c>
@@ -26966,7 +26966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>420</v>
       </c>
@@ -27061,7 +27061,7 @@
         <v>66376800000</v>
       </c>
     </row>
-    <row r="249" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>421</v>
       </c>
@@ -27156,7 +27156,7 @@
         <v>70556100000</v>
       </c>
     </row>
-    <row r="250" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>422</v>
       </c>
@@ -27251,7 +27251,7 @@
         <v>71170700000</v>
       </c>
     </row>
-    <row r="251" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>423</v>
       </c>
@@ -27346,7 +27346,7 @@
         <v>40293200000</v>
       </c>
     </row>
-    <row r="252" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>424</v>
       </c>
@@ -27441,7 +27441,7 @@
         <v>334588000000</v>
       </c>
     </row>
-    <row r="253" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>425</v>
       </c>
@@ -27536,7 +27536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>426</v>
       </c>
@@ -27631,7 +27631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>427</v>
       </c>
@@ -27726,7 +27726,7 @@
         <v>2105620000000</v>
       </c>
     </row>
-    <row r="256" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>428</v>
       </c>
@@ -27821,7 +27821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>429</v>
       </c>
@@ -27916,7 +27916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>430</v>
       </c>
@@ -28011,7 +28011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>431</v>
       </c>
@@ -28106,7 +28106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>432</v>
       </c>
@@ -28201,7 +28201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>433</v>
       </c>
@@ -28296,7 +28296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>434</v>
       </c>
@@ -28391,7 +28391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>435</v>
       </c>
@@ -28486,7 +28486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>436</v>
       </c>
@@ -28581,7 +28581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>437</v>
       </c>
@@ -28676,7 +28676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>438</v>
       </c>
@@ -28771,7 +28771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>439</v>
       </c>
@@ -28866,7 +28866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>440</v>
       </c>
@@ -28961,7 +28961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>441</v>
       </c>
@@ -29056,7 +29056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>442</v>
       </c>
@@ -29151,7 +29151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>443</v>
       </c>
@@ -29246,7 +29246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>444</v>
       </c>
@@ -29341,7 +29341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>445</v>
       </c>
@@ -29436,7 +29436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>446</v>
       </c>
@@ -29531,7 +29531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>447</v>
       </c>
@@ -29626,7 +29626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>448</v>
       </c>
@@ -29721,7 +29721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>449</v>
       </c>
@@ -29816,7 +29816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>450</v>
       </c>
@@ -29911,7 +29911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>451</v>
       </c>
@@ -30006,7 +30006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>452</v>
       </c>
@@ -30101,7 +30101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B281" s="38"/>
       <c r="C281" s="38"/>
       <c r="D281" s="38"/>
@@ -30133,7 +30133,7 @@
       <c r="AD281" s="38"/>
       <c r="AE281" s="38"/>
     </row>
-    <row r="282" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>167</v>
       </c>
@@ -30258,7 +30258,7 @@
         <v>118453820000000</v>
       </c>
     </row>
-    <row r="283" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B283" s="38"/>
       <c r="C283" s="38"/>
       <c r="D283" s="38"/>
@@ -30290,7 +30290,7 @@
       <c r="AD283" s="38"/>
       <c r="AE283" s="38"/>
     </row>
-    <row r="284" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B284" s="38"/>
       <c r="C284" s="38"/>
       <c r="D284" s="38"/>
@@ -30322,7 +30322,7 @@
       <c r="AD284" s="38"/>
       <c r="AE284" s="38"/>
     </row>
-    <row r="285" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B285" s="38"/>
       <c r="C285" s="38"/>
       <c r="D285" s="38"/>
@@ -30354,7 +30354,7 @@
       <c r="AD285" s="38"/>
       <c r="AE285" s="38"/>
     </row>
-    <row r="286" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B286" s="38"/>
       <c r="C286" s="38"/>
       <c r="D286" s="38"/>
@@ -30386,7 +30386,7 @@
       <c r="AD286" s="38"/>
       <c r="AE286" s="38"/>
     </row>
-    <row r="287" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B287" s="38"/>
       <c r="C287" s="38"/>
       <c r="D287" s="38"/>
@@ -30418,7 +30418,7 @@
       <c r="AD287" s="38"/>
       <c r="AE287" s="38"/>
     </row>
-    <row r="288" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:31" x14ac:dyDescent="0.35">
       <c r="B288" s="38"/>
       <c r="C288" s="38"/>
       <c r="D288" s="38"/>
@@ -30450,7 +30450,7 @@
       <c r="AD288" s="38"/>
       <c r="AE288" s="38"/>
     </row>
-    <row r="289" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B289" s="38"/>
       <c r="C289" s="38"/>
       <c r="D289" s="38"/>
@@ -30482,7 +30482,7 @@
       <c r="AD289" s="38"/>
       <c r="AE289" s="38"/>
     </row>
-    <row r="290" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B290" s="38"/>
       <c r="C290" s="38"/>
       <c r="D290" s="38"/>
@@ -30514,7 +30514,7 @@
       <c r="AD290" s="38"/>
       <c r="AE290" s="38"/>
     </row>
-    <row r="293" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B293" s="38"/>
       <c r="C293" s="38"/>
       <c r="D293" s="38"/>
@@ -30546,7 +30546,7 @@
       <c r="AD293" s="38"/>
       <c r="AE293" s="38"/>
     </row>
-    <row r="294" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B294" s="38"/>
       <c r="C294" s="38"/>
       <c r="D294" s="38"/>
@@ -30578,7 +30578,7 @@
       <c r="AD294" s="38"/>
       <c r="AE294" s="38"/>
     </row>
-    <row r="295" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B295" s="38"/>
       <c r="C295" s="38"/>
       <c r="D295" s="38"/>
@@ -30610,7 +30610,7 @@
       <c r="AD295" s="38"/>
       <c r="AE295" s="38"/>
     </row>
-    <row r="296" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B296" s="38"/>
       <c r="C296" s="38"/>
       <c r="D296" s="38"/>
@@ -30642,7 +30642,7 @@
       <c r="AD296" s="38"/>
       <c r="AE296" s="38"/>
     </row>
-    <row r="297" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B297" s="38"/>
       <c r="C297" s="38"/>
       <c r="D297" s="38"/>
@@ -30674,7 +30674,7 @@
       <c r="AD297" s="38"/>
       <c r="AE297" s="38"/>
     </row>
-    <row r="298" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B298" s="38"/>
       <c r="C298" s="38"/>
       <c r="D298" s="38"/>
@@ -30706,7 +30706,7 @@
       <c r="AD298" s="38"/>
       <c r="AE298" s="38"/>
     </row>
-    <row r="299" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B299" s="38"/>
       <c r="C299" s="38"/>
       <c r="D299" s="38"/>
@@ -30738,7 +30738,7 @@
       <c r="AD299" s="38"/>
       <c r="AE299" s="38"/>
     </row>
-    <row r="300" spans="2:31" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:31" x14ac:dyDescent="0.35">
       <c r="B300" s="38"/>
       <c r="C300" s="38"/>
       <c r="D300" s="38"/>
@@ -30781,12 +30781,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.85546875" customWidth="1"/>
+    <col min="1" max="1" width="29.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>169</v>
       </c>
@@ -30881,7 +30881,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -30976,7 +30976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -31071,7 +31071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -31166,7 +31166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -31261,7 +31261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -31356,7 +31356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -31451,7 +31451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -31546,7 +31546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -31641,7 +31641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -31736,7 +31736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -31831,7 +31831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -31926,7 +31926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -32021,7 +32021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -32116,7 +32116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -32211,7 +32211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -32306,7 +32306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -32401,7 +32401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -32496,7 +32496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -32591,7 +32591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -32686,7 +32686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -32781,7 +32781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -32876,7 +32876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -32971,7 +32971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -33066,7 +33066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -33161,7 +33161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -33267,14 +33267,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.85546875" customWidth="1"/>
+    <col min="1" max="1" width="44.81640625" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>169</v>
       </c>
@@ -33369,7 +33369,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -33464,7 +33464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -33559,7 +33559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -33654,7 +33654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -33749,7 +33749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -33844,7 +33844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -33939,7 +33939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -34034,7 +34034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -34129,7 +34129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -34254,7 +34254,7 @@
         <v>0.20635057803635587</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -34349,7 +34349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -34444,7 +34444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -34539,7 +34539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -34634,7 +34634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -34729,7 +34729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -34824,7 +34824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -34919,7 +34919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -35014,7 +35014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -35109,7 +35109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -35204,7 +35204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -35299,7 +35299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -35394,7 +35394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -35489,7 +35489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -35584,7 +35584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -35679,7 +35679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -35786,14 +35786,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.85546875" customWidth="1"/>
+    <col min="1" max="1" width="44.81640625" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>169</v>
       </c>
@@ -35888,7 +35888,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -35983,7 +35983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -36078,7 +36078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -36203,7 +36203,7 @@
         <v>0.2606786462633216</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -36298,7 +36298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -36393,7 +36393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -36488,7 +36488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -36583,7 +36583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -36678,7 +36678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -36803,7 +36803,7 @@
         <v>0.61297940852101807</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -36898,7 +36898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -36993,7 +36993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -37088,7 +37088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -37213,7 +37213,7 @@
         <v>0.15757487253490493</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -37338,7 +37338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -37433,7 +37433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -37528,7 +37528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -37623,7 +37623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -37718,7 +37718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -37813,7 +37813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -37908,7 +37908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -38003,7 +38003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -38098,7 +38098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -38193,7 +38193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -38288,7 +38288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
Correction to CCS achieved
</commit_message>
<xml_diff>
--- a/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
+++ b/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\ccs\NBICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E243723-5BA1-4981-9C22-BBBBBAB92F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6CAC593-305C-442B-8755-5B30E9F069F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-4770" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-29775" yWindow="210" windowWidth="23100" windowHeight="13620" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34134,124 +34134,94 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!B1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!B282</f>
         <v>0</v>
       </c>
       <c r="C10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!C1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!C282</f>
         <v>0</v>
       </c>
       <c r="D10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!D1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!D282</f>
         <v>0</v>
       </c>
       <c r="E10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!E1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!E282</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!F1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!F282</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!G1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!G282</f>
         <v>0</v>
       </c>
       <c r="H10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!H1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!H282</f>
         <v>0</v>
       </c>
       <c r="I10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!I1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!I282</f>
         <v>0</v>
       </c>
       <c r="J10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!J1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!J282</f>
         <v>0</v>
       </c>
       <c r="K10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!K1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!K282</f>
         <v>0</v>
       </c>
       <c r="L10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!L1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!L282</f>
-        <v>3.3837743903451734E-2</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!M1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!M282</f>
-        <v>6.8283995644973908E-2</v>
+        <v>0</v>
       </c>
       <c r="N10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!N1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!N282</f>
-        <v>0.10467368559617371</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!O1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!O282</f>
-        <v>0.14067318997097772</v>
-      </c>
-      <c r="P10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!P282</f>
-        <v>0.17800298250195254</v>
-      </c>
-      <c r="Q10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!Q282</f>
-        <v>0.18050682163530843</v>
-      </c>
-      <c r="R10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!R282</f>
-        <v>0.1829953861607781</v>
-      </c>
-      <c r="S10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!S282</f>
-        <v>0.18562188753311823</v>
-      </c>
-      <c r="T10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!T282</f>
-        <v>0.18721158898981899</v>
-      </c>
-      <c r="U10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!U282</f>
-        <v>0.18864204269445245</v>
-      </c>
-      <c r="V10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!V282</f>
-        <v>0.18976583463658167</v>
-      </c>
-      <c r="W10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!W282</f>
-        <v>0.18991320919812352</v>
-      </c>
-      <c r="X10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!X282</f>
-        <v>0.1922201773137226</v>
-      </c>
-      <c r="Y10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!Y282</f>
-        <v>0.19527195220967411</v>
-      </c>
-      <c r="Z10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!Z282</f>
-        <v>0.19862615357834532</v>
-      </c>
-      <c r="AA10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AA282</f>
-        <v>0.20302254172358283</v>
-      </c>
-      <c r="AB10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AB282</f>
-        <v>0.20439297406366849</v>
-      </c>
-      <c r="AC10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AC282</f>
-        <v>0.20235184503758905</v>
-      </c>
-      <c r="AD10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AD282</f>
-        <v>0.20345918052198869</v>
-      </c>
-      <c r="AE10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AE282</f>
-        <v>0.20635057803635587</v>
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.35">
@@ -36082,125 +36052,95 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B6</f>
-        <v>0.21277540815949841</v>
-      </c>
-      <c r="C4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C6</f>
-        <v>0.21508482860112188</v>
-      </c>
-      <c r="D4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D6</f>
-        <v>0.2226259619727412</v>
-      </c>
-      <c r="E4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E6</f>
-        <v>0.22358293585718725</v>
-      </c>
-      <c r="F4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F6</f>
-        <v>0.23490760158556884</v>
-      </c>
-      <c r="G4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G6</f>
-        <v>0.24109420727957445</v>
-      </c>
-      <c r="H4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H6</f>
-        <v>0.24367941014440636</v>
-      </c>
-      <c r="I4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I6</f>
-        <v>0.24505174430076465</v>
-      </c>
-      <c r="J4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J6</f>
-        <v>0.2455920252215717</v>
-      </c>
-      <c r="K4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K6</f>
-        <v>0.24856337097979461</v>
-      </c>
-      <c r="L4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L6</f>
-        <v>0.25169948413127824</v>
-      </c>
-      <c r="M4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M6</f>
-        <v>0.25593459706887262</v>
-      </c>
-      <c r="N4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N6</f>
-        <v>0.25933741490760942</v>
-      </c>
-      <c r="O4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O6</f>
-        <v>0.26007872787462005</v>
-      </c>
-      <c r="P4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P6</f>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="Q4" s="38">
-        <f>P4</f>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="R4" s="38">
-        <f t="shared" ref="R4:AE4" si="0">Q4</f>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="S4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="T4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="U4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="V4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="W4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="X4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="Y4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="Z4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AA4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AB4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AC4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AD4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AE4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.35">
@@ -36682,125 +36622,95 @@
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B12</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C12</f>
-        <v>1.7035952458279224E-2</v>
-      </c>
-      <c r="D10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D12</f>
-        <v>7.379540142338728E-2</v>
-      </c>
-      <c r="E10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E12</f>
-        <v>0.12978043460134511</v>
-      </c>
-      <c r="F10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F12</f>
-        <v>0.18340143676845078</v>
-      </c>
-      <c r="G10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G12</f>
-        <v>0.23726323944903455</v>
-      </c>
-      <c r="H10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H12</f>
-        <v>0.29179797708222832</v>
-      </c>
-      <c r="I10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I12</f>
-        <v>0.3465888690181968</v>
-      </c>
-      <c r="J10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J12</f>
-        <v>0.40293807245549862</v>
-      </c>
-      <c r="K10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K12</f>
-        <v>0.46127828033038998</v>
-      </c>
-      <c r="L10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L12</f>
-        <v>0.46428938925855379</v>
-      </c>
-      <c r="M10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M12</f>
-        <v>0.46892634931043969</v>
-      </c>
-      <c r="N10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N12</f>
-        <v>0.47908528156881697</v>
-      </c>
-      <c r="O10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O12</f>
-        <v>0.48916293796855054</v>
-      </c>
-      <c r="P10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P12</f>
-        <v>0.49657659767289786</v>
-      </c>
-      <c r="Q10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Q12</f>
-        <v>0.50296540850885785</v>
-      </c>
-      <c r="R10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!R12</f>
-        <v>0.51456524577321661</v>
-      </c>
-      <c r="S10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!S12</f>
-        <v>0.52416240494873922</v>
-      </c>
-      <c r="T10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!T12</f>
-        <v>0.5337411036527685</v>
-      </c>
-      <c r="U10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!U12</f>
-        <v>0.54446206562073074</v>
-      </c>
-      <c r="V10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!V12</f>
-        <v>0.55091923685396671</v>
-      </c>
-      <c r="W10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!W12</f>
-        <v>0.55490684703794002</v>
-      </c>
-      <c r="X10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!X12</f>
-        <v>0.5637005765733456</v>
-      </c>
-      <c r="Y10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Y12</f>
-        <v>0.56928750459812449</v>
-      </c>
-      <c r="Z10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Z12</f>
-        <v>0.57880294177833458</v>
-      </c>
-      <c r="AA10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AA12</f>
-        <v>0.58666244942241519</v>
-      </c>
-      <c r="AB10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AB12</f>
-        <v>0.60164854466283457</v>
-      </c>
-      <c r="AC10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AC12</f>
-        <v>0.61282270980178088</v>
-      </c>
-      <c r="AD10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AD12</f>
-        <v>0.61033926350690149</v>
-      </c>
-      <c r="AE10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AE12</f>
-        <v>0.61297940852101807</v>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.35">
@@ -37092,249 +37002,189 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B16</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C16</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D16</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E16</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F16</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G16</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H16</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I16</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J16</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K16</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L16</f>
-        <v>3.7752549827448745E-2</v>
-      </c>
-      <c r="M14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M16</f>
-        <v>7.4708155228358858E-2</v>
-      </c>
-      <c r="N14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N16</f>
-        <v>0.11118996808081458</v>
-      </c>
-      <c r="O14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O16</f>
-        <v>0.14768895426646664</v>
-      </c>
-      <c r="P14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P16</f>
-        <v>0.18326762641918265</v>
-      </c>
-      <c r="Q14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Q16</f>
-        <v>0.18033978663614653</v>
-      </c>
-      <c r="R14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!R16</f>
-        <v>0.17808339327690195</v>
-      </c>
-      <c r="S14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!S16</f>
-        <v>0.1763327754868112</v>
-      </c>
-      <c r="T14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!T16</f>
-        <v>0.17447664100800267</v>
-      </c>
-      <c r="U14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!U16</f>
-        <v>0.17311570475476731</v>
-      </c>
-      <c r="V14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!V16</f>
-        <v>0.17130392343865253</v>
-      </c>
-      <c r="W14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!W16</f>
-        <v>0.16913551934449236</v>
-      </c>
-      <c r="X14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!X16</f>
-        <v>0.16744848986765473</v>
-      </c>
-      <c r="Y14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Y16</f>
-        <v>0.16665994536910525</v>
-      </c>
-      <c r="Z14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Z16</f>
-        <v>0.16493855533002394</v>
-      </c>
-      <c r="AA14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AA16</f>
-        <v>0.16304908364650231</v>
-      </c>
-      <c r="AB14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AB16</f>
-        <v>0.1615604183547267</v>
-      </c>
-      <c r="AC14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AC16</f>
-        <v>0.1600399890937497</v>
-      </c>
-      <c r="AD14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AD16</f>
-        <v>0.15881712441055912</v>
-      </c>
-      <c r="AE14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AE16</f>
-        <v>0.15757487253490493</v>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+      <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B17</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C17</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D17</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E17</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F17</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G17</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H17</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I17</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J17</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K17</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L17</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M17</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N17</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O17</f>
-        <v>0</v>
-      </c>
-      <c r="P15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P17</f>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Q17</f>
-        <v>0</v>
-      </c>
-      <c r="R15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!R17</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!S17</f>
-        <v>0</v>
-      </c>
-      <c r="T15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!T17</f>
-        <v>0</v>
-      </c>
-      <c r="U15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!U17</f>
-        <v>0</v>
-      </c>
-      <c r="V15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!V17</f>
-        <v>0</v>
-      </c>
-      <c r="W15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!W17</f>
-        <v>0</v>
-      </c>
-      <c r="X15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!X17</f>
-        <v>0</v>
-      </c>
-      <c r="Y15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Y17</f>
-        <v>0</v>
-      </c>
-      <c r="Z15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Z17</f>
-        <v>0</v>
-      </c>
-      <c r="AA15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AA17</f>
-        <v>0</v>
-      </c>
-      <c r="AB15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AB17</f>
-        <v>0</v>
-      </c>
-      <c r="AC15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AC17</f>
-        <v>0</v>
-      </c>
-      <c r="AD15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AD17</f>
-        <v>0</v>
-      </c>
-      <c r="AE15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AE17</f>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated DLIM and TLIM to newest OECD data, CCS correction
</commit_message>
<xml_diff>
--- a/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
+++ b/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\ccs\NBICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E243723-5BA1-4981-9C22-BBBBBAB92F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6CAC593-305C-442B-8755-5B30E9F069F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-4770" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-29775" yWindow="210" windowWidth="23100" windowHeight="13620" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34134,124 +34134,94 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!B1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!B282</f>
         <v>0</v>
       </c>
       <c r="C10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!C1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!C282</f>
         <v>0</v>
       </c>
       <c r="D10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!D1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!D282</f>
         <v>0</v>
       </c>
       <c r="E10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!E1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!E282</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!F1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!F282</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!G1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!G282</f>
         <v>0</v>
       </c>
       <c r="H10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!H1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!H282</f>
         <v>0</v>
       </c>
       <c r="I10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!I1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!I282</f>
         <v>0</v>
       </c>
       <c r="J10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!J1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!J282</f>
         <v>0</v>
       </c>
       <c r="K10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!K1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!K282</f>
         <v>0</v>
       </c>
       <c r="L10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!L1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!L282</f>
-        <v>3.3837743903451734E-2</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!M1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!M282</f>
-        <v>6.8283995644973908E-2</v>
+        <v>0</v>
       </c>
       <c r="N10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!N1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!N282</f>
-        <v>0.10467368559617371</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!O1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!O282</f>
-        <v>0.14067318997097772</v>
-      </c>
-      <c r="P10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!P282</f>
-        <v>0.17800298250195254</v>
-      </c>
-      <c r="Q10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!Q282</f>
-        <v>0.18050682163530843</v>
-      </c>
-      <c r="R10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!R282</f>
-        <v>0.1829953861607781</v>
-      </c>
-      <c r="S10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!S282</f>
-        <v>0.18562188753311823</v>
-      </c>
-      <c r="T10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!T282</f>
-        <v>0.18721158898981899</v>
-      </c>
-      <c r="U10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!U282</f>
-        <v>0.18864204269445245</v>
-      </c>
-      <c r="V10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!V282</f>
-        <v>0.18976583463658167</v>
-      </c>
-      <c r="W10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!W282</f>
-        <v>0.18991320919812352</v>
-      </c>
-      <c r="X10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!X282</f>
-        <v>0.1922201773137226</v>
-      </c>
-      <c r="Y10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!Y282</f>
-        <v>0.19527195220967411</v>
-      </c>
-      <c r="Z10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!Z282</f>
-        <v>0.19862615357834532</v>
-      </c>
-      <c r="AA10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AA282</f>
-        <v>0.20302254172358283</v>
-      </c>
-      <c r="AB10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AB282</f>
-        <v>0.20439297406366849</v>
-      </c>
-      <c r="AC10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AC282</f>
-        <v>0.20235184503758905</v>
-      </c>
-      <c r="AD10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AD282</f>
-        <v>0.20345918052198869</v>
-      </c>
-      <c r="AE10" s="38">
-        <f>(MAX(TREND('Current and Planned Capacity'!$C$35:$D$35,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-energyEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12)/'BAU Emissions'!AE282</f>
-        <v>0.20635057803635587</v>
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.35">
@@ -36082,125 +36052,95 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B6</f>
-        <v>0.21277540815949841</v>
-      </c>
-      <c r="C4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C6</f>
-        <v>0.21508482860112188</v>
-      </c>
-      <c r="D4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D6</f>
-        <v>0.2226259619727412</v>
-      </c>
-      <c r="E4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E6</f>
-        <v>0.22358293585718725</v>
-      </c>
-      <c r="F4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F6</f>
-        <v>0.23490760158556884</v>
-      </c>
-      <c r="G4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G6</f>
-        <v>0.24109420727957445</v>
-      </c>
-      <c r="H4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H6</f>
-        <v>0.24367941014440636</v>
-      </c>
-      <c r="I4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I6</f>
-        <v>0.24505174430076465</v>
-      </c>
-      <c r="J4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J6</f>
-        <v>0.2455920252215717</v>
-      </c>
-      <c r="K4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K6</f>
-        <v>0.24856337097979461</v>
-      </c>
-      <c r="L4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L6</f>
-        <v>0.25169948413127824</v>
-      </c>
-      <c r="M4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M6</f>
-        <v>0.25593459706887262</v>
-      </c>
-      <c r="N4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N6</f>
-        <v>0.25933741490760942</v>
-      </c>
-      <c r="O4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O6</f>
-        <v>0.26007872787462005</v>
-      </c>
-      <c r="P4" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$29:$C$29,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P6</f>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="Q4" s="38">
-        <f>P4</f>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="R4" s="38">
-        <f t="shared" ref="R4:AE4" si="0">Q4</f>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="S4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="T4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="U4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="V4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="W4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="X4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="Y4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="Z4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AA4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AB4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AC4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AD4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
-      </c>
-      <c r="AE4" s="38">
-        <f t="shared" si="0"/>
-        <v>0.2606786462633216</v>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.35">
@@ -36682,125 +36622,95 @@
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B12</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C12</f>
-        <v>1.7035952458279224E-2</v>
-      </c>
-      <c r="D10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D12</f>
-        <v>7.379540142338728E-2</v>
-      </c>
-      <c r="E10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E12</f>
-        <v>0.12978043460134511</v>
-      </c>
-      <c r="F10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F12</f>
-        <v>0.18340143676845078</v>
-      </c>
-      <c r="G10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G12</f>
-        <v>0.23726323944903455</v>
-      </c>
-      <c r="H10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H12</f>
-        <v>0.29179797708222832</v>
-      </c>
-      <c r="I10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I12</f>
-        <v>0.3465888690181968</v>
-      </c>
-      <c r="J10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$36:$C$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J12</f>
-        <v>0.40293807245549862</v>
-      </c>
-      <c r="K10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K12</f>
-        <v>0.46127828033038998</v>
-      </c>
-      <c r="L10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L12</f>
-        <v>0.46428938925855379</v>
-      </c>
-      <c r="M10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M12</f>
-        <v>0.46892634931043969</v>
-      </c>
-      <c r="N10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N12</f>
-        <v>0.47908528156881697</v>
-      </c>
-      <c r="O10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O12</f>
-        <v>0.48916293796855054</v>
-      </c>
-      <c r="P10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P12</f>
-        <v>0.49657659767289786</v>
-      </c>
-      <c r="Q10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Q12</f>
-        <v>0.50296540850885785</v>
-      </c>
-      <c r="R10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!R12</f>
-        <v>0.51456524577321661</v>
-      </c>
-      <c r="S10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!S12</f>
-        <v>0.52416240494873922</v>
-      </c>
-      <c r="T10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!T12</f>
-        <v>0.5337411036527685</v>
-      </c>
-      <c r="U10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!U12</f>
-        <v>0.54446206562073074</v>
-      </c>
-      <c r="V10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!V12</f>
-        <v>0.55091923685396671</v>
-      </c>
-      <c r="W10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!W12</f>
-        <v>0.55490684703794002</v>
-      </c>
-      <c r="X10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!X12</f>
-        <v>0.5637005765733456</v>
-      </c>
-      <c r="Y10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Y12</f>
-        <v>0.56928750459812449</v>
-      </c>
-      <c r="Z10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Z12</f>
-        <v>0.57880294177833458</v>
-      </c>
-      <c r="AA10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AA12</f>
-        <v>0.58666244942241519</v>
-      </c>
-      <c r="AB10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AB12</f>
-        <v>0.60164854466283457</v>
-      </c>
-      <c r="AC10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AC12</f>
-        <v>0.61282270980178088</v>
-      </c>
-      <c r="AD10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AD12</f>
-        <v>0.61033926350690149</v>
-      </c>
-      <c r="AE10" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$36:$D$36,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AE12</f>
-        <v>0.61297940852101807</v>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.35">
@@ -37092,249 +37002,189 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B16</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C16</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D16</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E16</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F16</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G16</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H16</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I16</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J16</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$40:$C$40,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K16</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L16</f>
-        <v>3.7752549827448745E-2</v>
-      </c>
-      <c r="M14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M16</f>
-        <v>7.4708155228358858E-2</v>
-      </c>
-      <c r="N14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N16</f>
-        <v>0.11118996808081458</v>
-      </c>
-      <c r="O14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O16</f>
-        <v>0.14768895426646664</v>
-      </c>
-      <c r="P14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P16</f>
-        <v>0.18326762641918265</v>
-      </c>
-      <c r="Q14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Q16</f>
-        <v>0.18033978663614653</v>
-      </c>
-      <c r="R14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!R16</f>
-        <v>0.17808339327690195</v>
-      </c>
-      <c r="S14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!S16</f>
-        <v>0.1763327754868112</v>
-      </c>
-      <c r="T14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!T16</f>
-        <v>0.17447664100800267</v>
-      </c>
-      <c r="U14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!U16</f>
-        <v>0.17311570475476731</v>
-      </c>
-      <c r="V14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!V16</f>
-        <v>0.17130392343865253</v>
-      </c>
-      <c r="W14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!W16</f>
-        <v>0.16913551934449236</v>
-      </c>
-      <c r="X14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!X16</f>
-        <v>0.16744848986765473</v>
-      </c>
-      <c r="Y14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Y16</f>
-        <v>0.16665994536910525</v>
-      </c>
-      <c r="Z14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Z16</f>
-        <v>0.16493855533002394</v>
-      </c>
-      <c r="AA14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AA16</f>
-        <v>0.16304908364650231</v>
-      </c>
-      <c r="AB14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AB16</f>
-        <v>0.1615604183547267</v>
-      </c>
-      <c r="AC14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AC16</f>
-        <v>0.1600399890937497</v>
-      </c>
-      <c r="AD14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AD16</f>
-        <v>0.15881712441055912</v>
-      </c>
-      <c r="AE14" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$40:$D$40,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AE16</f>
-        <v>0.15757487253490493</v>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+      <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!B$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!B17</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!C$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!C17</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!D$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!D17</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!E$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!E17</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!F$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!F17</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!G$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!G17</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!H$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!H17</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!I$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!I17</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!J$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!J17</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$B$41:$C$41,'Current and Planned Capacity'!$B$26:$C$26,'NBICP-FoCPAbI-processEmis'!K$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!K17</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!L$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!L17</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!M$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!M17</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!N$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!N17</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!O$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!O17</f>
-        <v>0</v>
-      </c>
-      <c r="P15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!P17</f>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Q17</f>
-        <v>0</v>
-      </c>
-      <c r="R15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!R17</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!S17</f>
-        <v>0</v>
-      </c>
-      <c r="T15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!T17</f>
-        <v>0</v>
-      </c>
-      <c r="U15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!U17</f>
-        <v>0</v>
-      </c>
-      <c r="V15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!V17</f>
-        <v>0</v>
-      </c>
-      <c r="W15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!W17</f>
-        <v>0</v>
-      </c>
-      <c r="X15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!X17</f>
-        <v>0</v>
-      </c>
-      <c r="Y15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Y17</f>
-        <v>0</v>
-      </c>
-      <c r="Z15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!Z17</f>
-        <v>0</v>
-      </c>
-      <c r="AA15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AA17</f>
-        <v>0</v>
-      </c>
-      <c r="AB15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AB17</f>
-        <v>0</v>
-      </c>
-      <c r="AC15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AC17</f>
-        <v>0</v>
-      </c>
-      <c r="AD15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AD17</f>
-        <v>0</v>
-      </c>
-      <c r="AE15" s="38">
-        <f>MAX(TREND('Current and Planned Capacity'!$C$41:$D$41,'Current and Planned Capacity'!$C$26:$D$26,'NBICP-FoCPAbI-processEmis'!$P$1),0)*'Capacity Factor Data'!$A$45*10^12/'BAU Emissions'!AE17</f>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
         <v>0</v>
       </c>
     </row>

</xml_diff>